<commit_message>
Mise à jour dashboard
</commit_message>
<xml_diff>
--- a/donnees_avicole_bd.xlsx
+++ b/donnees_avicole_bd.xlsx
@@ -1,16 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25831"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30117"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\Dashboard\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27A9D10F-9DFD-479B-BF05-7A7C855D5195}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="11_B68137C8777E7AAABD29645CAADFCB6A974F3387" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FA0D029B-7B2A-4B10-8FA2-342B41A34CDB}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="journalier" sheetId="1" r:id="rId1"/>
@@ -30,6 +25,7 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -37,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="118">
   <si>
     <t>date</t>
   </si>
@@ -297,6 +293,9 @@
     <t>taux_marge_sur_couts_variables_pct</t>
   </si>
   <si>
+    <t>investissements_globaux_fcfa</t>
+  </si>
+  <si>
     <t>COB</t>
   </si>
   <si>
@@ -325,6 +324,69 @@
   </si>
   <si>
     <t>prix_total</t>
+  </si>
+  <si>
+    <t>acheteur</t>
+  </si>
+  <si>
+    <t>Jean</t>
+  </si>
+  <si>
+    <t>Babacar</t>
+  </si>
+  <si>
+    <t>Wade</t>
+  </si>
+  <si>
+    <t>jean</t>
+  </si>
+  <si>
+    <t>contact de Jean</t>
+  </si>
+  <si>
+    <t>Fatima association</t>
+  </si>
+  <si>
+    <t>neuveu de Jean</t>
+  </si>
+  <si>
+    <t>Kebe</t>
+  </si>
+  <si>
+    <t>INIS- Moustapha Dakar</t>
+  </si>
+  <si>
+    <t>Mme Fatima (association)</t>
+  </si>
+  <si>
+    <t>Cheikh guediawaye -INIS</t>
+  </si>
+  <si>
+    <t>djiby Guinar</t>
+  </si>
+  <si>
+    <t>Mouhamed</t>
+  </si>
+  <si>
+    <t>Baye Fall</t>
+  </si>
+  <si>
+    <t>Khadim- Nguirane</t>
+  </si>
+  <si>
+    <t>colonel gaye</t>
+  </si>
+  <si>
+    <t>Babacar ferme</t>
+  </si>
+  <si>
+    <t>Khadim</t>
+  </si>
+  <si>
+    <t>Khadim-Nguirane</t>
+  </si>
+  <si>
+    <t>Nguirane</t>
   </si>
 </sst>
 </file>
@@ -334,7 +396,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -346,13 +408,6 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -390,13 +445,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -700,17 +754,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N181"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="18.28515625" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.5703125" customWidth="1"/>
-    <col min="9" max="9" width="14.85546875" customWidth="1"/>
-    <col min="10" max="11" width="16.42578125" customWidth="1"/>
-    <col min="12" max="12" width="21.7109375" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -754,7 +800,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14">
       <c r="A2" s="2">
         <v>45934</v>
       </c>
@@ -792,7 +838,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14">
       <c r="A3" s="2">
         <v>45935</v>
       </c>
@@ -824,7 +870,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14">
       <c r="A4" s="2">
         <v>45936</v>
       </c>
@@ -856,7 +902,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14">
       <c r="A5" s="2">
         <v>45937</v>
       </c>
@@ -888,7 +934,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14">
       <c r="A6" s="2">
         <v>45938</v>
       </c>
@@ -920,7 +966,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14">
       <c r="A7" s="2">
         <v>45939</v>
       </c>
@@ -961,7 +1007,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14">
       <c r="A8" s="2">
         <v>45940</v>
       </c>
@@ -993,7 +1039,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14">
       <c r="A9" s="2">
         <v>45941</v>
       </c>
@@ -1028,7 +1074,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14">
       <c r="A10" s="2">
         <v>45942</v>
       </c>
@@ -1072,7 +1118,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14">
       <c r="A11" s="2">
         <v>45943</v>
       </c>
@@ -1104,7 +1150,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14">
       <c r="A12" s="2">
         <v>45944</v>
       </c>
@@ -1136,7 +1182,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14">
       <c r="A13" s="2">
         <v>45945</v>
       </c>
@@ -1171,7 +1217,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14">
       <c r="A14" s="2">
         <v>45946</v>
       </c>
@@ -1203,7 +1249,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14">
       <c r="A15" s="2">
         <v>45947</v>
       </c>
@@ -1247,7 +1293,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14">
       <c r="A16" s="2">
         <v>45948</v>
       </c>
@@ -1282,7 +1328,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14">
       <c r="A17" s="2">
         <v>45949</v>
       </c>
@@ -1314,7 +1360,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14">
       <c r="A18" s="2">
         <v>45950</v>
       </c>
@@ -1349,11 +1395,11 @@
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14">
       <c r="A19" s="2">
         <v>45951</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" t="s">
         <v>20</v>
       </c>
       <c r="C19">
@@ -1384,11 +1430,11 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14">
       <c r="A20" s="2">
         <v>45952</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" t="s">
         <v>20</v>
       </c>
       <c r="C20">
@@ -1419,7 +1465,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14">
       <c r="A21" s="2">
         <v>45953</v>
       </c>
@@ -1451,7 +1497,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14">
       <c r="A22" s="2">
         <v>45954</v>
       </c>
@@ -1495,7 +1541,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14">
       <c r="A23" s="2">
         <v>45955</v>
       </c>
@@ -1527,7 +1573,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14">
       <c r="A24" s="2">
         <v>45956</v>
       </c>
@@ -1559,7 +1605,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14">
       <c r="A25" s="2">
         <v>45957</v>
       </c>
@@ -1591,7 +1637,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14">
       <c r="A26" s="2">
         <v>45958</v>
       </c>
@@ -1623,7 +1669,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14">
       <c r="A27" s="2">
         <v>45959</v>
       </c>
@@ -1655,7 +1701,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14">
       <c r="A28" s="2">
         <v>45960</v>
       </c>
@@ -1687,7 +1733,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14">
       <c r="A29" s="2">
         <v>45961</v>
       </c>
@@ -1731,7 +1777,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14">
       <c r="A30" s="2">
         <v>45962</v>
       </c>
@@ -1763,7 +1809,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14">
       <c r="A31" s="2">
         <v>45963</v>
       </c>
@@ -1801,7 +1847,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14">
       <c r="A32" s="2">
         <v>45964</v>
       </c>
@@ -1833,7 +1879,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14">
       <c r="A33" s="2">
         <v>45965</v>
       </c>
@@ -1865,7 +1911,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14">
       <c r="A34" s="2">
         <v>45966</v>
       </c>
@@ -1897,7 +1943,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14">
       <c r="A35" s="2">
         <v>45967</v>
       </c>
@@ -1929,7 +1975,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14">
       <c r="A36" s="2">
         <v>45968</v>
       </c>
@@ -1970,7 +2016,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14">
       <c r="A37" s="2">
         <v>45969</v>
       </c>
@@ -2002,7 +2048,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:14">
       <c r="A38" s="2">
         <v>45970</v>
       </c>
@@ -2037,7 +2083,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:14">
       <c r="A39" s="2">
         <v>45971</v>
       </c>
@@ -2069,7 +2115,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:14">
       <c r="A40" s="2">
         <v>45972</v>
       </c>
@@ -2101,7 +2147,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:14">
       <c r="A41" s="2">
         <v>45973</v>
       </c>
@@ -2133,7 +2179,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:14">
       <c r="A42" s="2">
         <v>45974</v>
       </c>
@@ -2165,7 +2211,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:14">
       <c r="A43" s="2">
         <v>45975</v>
       </c>
@@ -2200,7 +2246,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:14">
       <c r="A44" s="2">
         <v>45976</v>
       </c>
@@ -2232,7 +2278,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:14">
       <c r="A45" s="2">
         <v>45977</v>
       </c>
@@ -2264,7 +2310,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:14">
       <c r="A46" s="2">
         <v>45978</v>
       </c>
@@ -2299,7 +2345,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:14">
       <c r="A47" s="2">
         <v>45979</v>
       </c>
@@ -2331,7 +2377,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:14">
       <c r="A48" s="2">
         <v>45980</v>
       </c>
@@ -2363,7 +2409,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:14">
       <c r="A49" s="2">
         <v>45981</v>
       </c>
@@ -2395,7 +2441,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:14">
       <c r="A50" s="2">
         <v>45982</v>
       </c>
@@ -2427,7 +2473,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:14">
       <c r="A51" s="2">
         <v>45983</v>
       </c>
@@ -2459,7 +2505,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:14">
       <c r="A52" s="2">
         <v>45984</v>
       </c>
@@ -2494,7 +2540,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:14">
       <c r="A53" s="2">
         <v>45985</v>
       </c>
@@ -2526,7 +2572,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:14">
       <c r="A54" s="2">
         <v>45986</v>
       </c>
@@ -2558,7 +2604,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:14">
       <c r="A55" s="2">
         <v>45987</v>
       </c>
@@ -2590,7 +2636,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:14">
       <c r="A56" s="2">
         <v>45988</v>
       </c>
@@ -2622,7 +2668,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:14">
       <c r="A57" s="2">
         <v>45989</v>
       </c>
@@ -2654,7 +2700,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:14">
       <c r="A58" s="2">
         <v>45990</v>
       </c>
@@ -2686,7 +2732,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:14">
       <c r="A59" s="2">
         <v>45991</v>
       </c>
@@ -2718,7 +2764,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:14">
       <c r="A60" s="2">
         <v>45992</v>
       </c>
@@ -2750,7 +2796,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:14">
       <c r="A61" s="2">
         <v>45993</v>
       </c>
@@ -2782,7 +2828,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:14">
       <c r="A62" s="2">
         <v>45995</v>
       </c>
@@ -2820,7 +2866,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:14">
       <c r="A63" s="2">
         <v>45996</v>
       </c>
@@ -2849,7 +2895,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:14">
       <c r="A64" s="2">
         <v>45997</v>
       </c>
@@ -2878,7 +2924,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:14">
       <c r="A65" s="2">
         <v>45998</v>
       </c>
@@ -2907,7 +2953,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:14">
       <c r="A66" s="2">
         <v>45999</v>
       </c>
@@ -2936,7 +2982,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:14">
       <c r="A67" s="2">
         <v>46000</v>
       </c>
@@ -2968,7 +3014,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:14">
       <c r="A68" s="2">
         <v>46001</v>
       </c>
@@ -2997,7 +3043,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:14">
       <c r="A69" s="2">
         <v>46002</v>
       </c>
@@ -3026,7 +3072,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:14">
       <c r="A70" s="2">
         <v>46003</v>
       </c>
@@ -3067,7 +3113,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:14">
       <c r="A71" s="2">
         <v>46004</v>
       </c>
@@ -3096,7 +3142,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:14">
       <c r="A72" s="2">
         <v>46005</v>
       </c>
@@ -3125,7 +3171,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:14">
       <c r="A73" s="2">
         <v>46006</v>
       </c>
@@ -3157,7 +3203,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:14">
       <c r="A74" s="2">
         <v>46007</v>
       </c>
@@ -3186,7 +3232,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:14">
       <c r="A75" s="2">
         <v>46008</v>
       </c>
@@ -3221,7 +3267,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="76" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:14">
       <c r="A76" s="2">
         <v>46009</v>
       </c>
@@ -3253,7 +3299,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:14">
       <c r="A77" s="2">
         <v>46010</v>
       </c>
@@ -3294,7 +3340,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="78" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:14">
       <c r="A78" s="2">
         <v>46011</v>
       </c>
@@ -3326,11 +3372,11 @@
         <v>26</v>
       </c>
     </row>
-    <row r="79" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:14">
       <c r="A79" s="2">
         <v>46012</v>
       </c>
-      <c r="B79" s="3" t="s">
+      <c r="B79" t="s">
         <v>20</v>
       </c>
       <c r="C79">
@@ -3358,11 +3404,11 @@
         <v>26</v>
       </c>
     </row>
-    <row r="80" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:14">
       <c r="A80" s="2">
         <v>46013</v>
       </c>
-      <c r="B80" s="3" t="s">
+      <c r="B80" t="s">
         <v>20</v>
       </c>
       <c r="C80">
@@ -3390,7 +3436,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="81" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:14">
       <c r="A81" s="2">
         <v>46014</v>
       </c>
@@ -3419,7 +3465,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="82" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:14">
       <c r="A82" s="2">
         <v>46015</v>
       </c>
@@ -3451,7 +3497,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="83" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:14">
       <c r="A83" s="2">
         <v>46016</v>
       </c>
@@ -3483,7 +3529,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="84" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:14">
       <c r="A84" s="2">
         <v>46017</v>
       </c>
@@ -3521,7 +3567,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="85" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:14">
       <c r="A85" s="2">
         <v>46018</v>
       </c>
@@ -3550,7 +3596,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="86" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:14">
       <c r="A86" s="2">
         <v>46019</v>
       </c>
@@ -3579,7 +3625,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="87" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:14">
       <c r="A87" s="2">
         <v>46020</v>
       </c>
@@ -3608,7 +3654,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="88" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:14">
       <c r="A88" s="2">
         <v>46021</v>
       </c>
@@ -3637,7 +3683,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="89" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:14">
       <c r="A89" s="2">
         <v>46022</v>
       </c>
@@ -3669,7 +3715,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="90" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:14">
       <c r="A90" s="2">
         <v>46023</v>
       </c>
@@ -3701,7 +3747,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="91" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:14">
       <c r="A91" s="2">
         <v>46024</v>
       </c>
@@ -3742,7 +3788,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="92" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:14">
       <c r="A92" s="2">
         <v>46025</v>
       </c>
@@ -3771,7 +3817,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="93" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:14">
       <c r="A93" s="2">
         <v>46026</v>
       </c>
@@ -3800,7 +3846,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="94" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:14">
       <c r="A94" s="2">
         <v>46027</v>
       </c>
@@ -3829,7 +3875,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="95" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:14">
       <c r="A95" s="2">
         <v>46028</v>
       </c>
@@ -3858,7 +3904,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="96" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:14">
       <c r="A96" s="2">
         <v>46029</v>
       </c>
@@ -3887,7 +3933,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="97" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:14">
       <c r="A97" s="2">
         <v>46030</v>
       </c>
@@ -3916,7 +3962,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="98" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:14">
       <c r="A98" s="2">
         <v>46031</v>
       </c>
@@ -3957,7 +4003,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="99" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:14">
       <c r="A99" s="2">
         <v>46032</v>
       </c>
@@ -3986,7 +4032,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="100" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:14">
       <c r="A100" s="2">
         <v>46033</v>
       </c>
@@ -4015,7 +4061,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="101" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:14">
       <c r="A101" s="2">
         <v>46034</v>
       </c>
@@ -4044,7 +4090,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="102" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:14">
       <c r="A102" s="2">
         <v>46035</v>
       </c>
@@ -4073,7 +4119,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="103" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:14">
       <c r="A103" s="2">
         <v>46036</v>
       </c>
@@ -4105,7 +4151,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="104" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:14">
       <c r="A104" s="2">
         <v>46037</v>
       </c>
@@ -4134,7 +4180,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="105" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:14">
       <c r="A105" s="2">
         <v>46038</v>
       </c>
@@ -4163,7 +4209,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="106" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:14">
       <c r="A106" s="2">
         <v>46039</v>
       </c>
@@ -4195,7 +4241,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="107" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:14">
       <c r="A107" s="2">
         <v>46040</v>
       </c>
@@ -4224,7 +4270,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="108" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:14">
       <c r="A108" s="2">
         <v>46041</v>
       </c>
@@ -4253,7 +4299,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="109" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:14">
       <c r="A109" s="2">
         <v>46042</v>
       </c>
@@ -4282,7 +4328,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="110" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:14">
       <c r="A110" s="2">
         <v>46043</v>
       </c>
@@ -4311,7 +4357,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="111" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:14">
       <c r="A111" s="2">
         <v>46044</v>
       </c>
@@ -4340,7 +4386,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="112" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:14">
       <c r="A112" s="2">
         <v>46045</v>
       </c>
@@ -4369,7 +4415,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="113" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:14">
       <c r="A113" s="2">
         <v>46046</v>
       </c>
@@ -4398,7 +4444,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="114" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:14">
       <c r="A114" s="2">
         <v>46047</v>
       </c>
@@ -4427,7 +4473,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="115" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:14">
       <c r="A115" s="2">
         <v>46048</v>
       </c>
@@ -4456,7 +4502,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="116" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:14">
       <c r="A116" s="2">
         <v>46049</v>
       </c>
@@ -4485,7 +4531,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="117" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:14">
       <c r="A117" s="2">
         <v>46050</v>
       </c>
@@ -4514,7 +4560,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="118" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:14">
       <c r="A118" s="2">
         <v>46051</v>
       </c>
@@ -4543,7 +4589,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="119" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:14">
       <c r="A119" s="2">
         <v>46052</v>
       </c>
@@ -4572,7 +4618,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="120" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:14">
       <c r="A120" s="2">
         <v>46053</v>
       </c>
@@ -4601,7 +4647,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="121" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:14">
       <c r="A121" s="2">
         <v>46054</v>
       </c>
@@ -4630,7 +4676,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="122" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:14">
       <c r="A122" s="2">
         <v>46027</v>
       </c>
@@ -4662,7 +4708,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="123" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:14">
       <c r="A123" s="2">
         <v>46028</v>
       </c>
@@ -4691,7 +4737,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="124" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:14">
       <c r="A124" s="2">
         <v>46029</v>
       </c>
@@ -4720,7 +4766,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="125" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:14">
       <c r="A125" s="2">
         <v>46030</v>
       </c>
@@ -4749,7 +4795,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="126" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:14">
       <c r="A126" s="2">
         <v>46031</v>
       </c>
@@ -4784,7 +4830,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="127" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:14">
       <c r="A127" s="2">
         <v>46032</v>
       </c>
@@ -4816,7 +4862,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="128" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:14">
       <c r="A128" s="2">
         <v>46033</v>
       </c>
@@ -4845,7 +4891,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="129" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:14">
       <c r="A129" s="2">
         <v>46034</v>
       </c>
@@ -4874,7 +4920,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="130" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:14">
       <c r="A130" s="2">
         <v>46035</v>
       </c>
@@ -4909,7 +4955,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="131" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:14">
       <c r="A131" s="2">
         <v>46036</v>
       </c>
@@ -4938,7 +4984,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="132" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:14">
       <c r="A132" s="2">
         <v>46037</v>
       </c>
@@ -4967,7 +5013,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="133" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:14">
       <c r="A133" s="2">
         <v>46038</v>
       </c>
@@ -4999,7 +5045,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="134" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:14">
       <c r="A134" s="2">
         <v>46039</v>
       </c>
@@ -5028,7 +5074,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="135" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:14">
       <c r="A135" s="2">
         <v>46040</v>
       </c>
@@ -5063,7 +5109,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="136" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:14">
       <c r="A136" s="2">
         <v>46041</v>
       </c>
@@ -5095,7 +5141,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="137" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:14">
       <c r="A137" s="2">
         <v>46042</v>
       </c>
@@ -5130,7 +5176,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="138" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:14">
       <c r="A138" s="2">
         <v>46043</v>
       </c>
@@ -5162,11 +5208,11 @@
         <v>28</v>
       </c>
     </row>
-    <row r="139" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:14">
       <c r="A139" s="2">
         <v>46044</v>
       </c>
-      <c r="B139" s="3" t="s">
+      <c r="B139" t="s">
         <v>20</v>
       </c>
       <c r="C139">
@@ -5194,11 +5240,11 @@
         <v>28</v>
       </c>
     </row>
-    <row r="140" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:14">
       <c r="A140" s="2">
         <v>46045</v>
       </c>
-      <c r="B140" s="3" t="s">
+      <c r="B140" t="s">
         <v>20</v>
       </c>
       <c r="C140">
@@ -5226,11 +5272,11 @@
         <v>28</v>
       </c>
     </row>
-    <row r="141" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:14">
       <c r="A141" s="2">
         <v>46046</v>
       </c>
-      <c r="B141" s="3" t="s">
+      <c r="B141" t="s">
         <v>20</v>
       </c>
       <c r="C141">
@@ -5264,7 +5310,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="142" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:14">
       <c r="A142" s="2">
         <v>46047</v>
       </c>
@@ -5296,7 +5342,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="143" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:14">
       <c r="A143" s="2">
         <v>46048</v>
       </c>
@@ -5334,7 +5380,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="144" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:14">
       <c r="A144" s="2">
         <v>46049</v>
       </c>
@@ -5366,7 +5412,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="145" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:14">
       <c r="A145" s="2">
         <v>46050</v>
       </c>
@@ -5395,7 +5441,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="146" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:14">
       <c r="A146" s="2">
         <v>46051</v>
       </c>
@@ -5424,7 +5470,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="147" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:14">
       <c r="A147" s="2">
         <v>46052</v>
       </c>
@@ -5453,7 +5499,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="148" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:14">
       <c r="A148" s="2">
         <v>46053</v>
       </c>
@@ -5482,7 +5528,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="149" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:14">
       <c r="A149" s="2">
         <v>46054</v>
       </c>
@@ -5511,7 +5557,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="150" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:14">
       <c r="A150" s="2">
         <v>46055</v>
       </c>
@@ -5552,7 +5598,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="151" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:14">
       <c r="A151" s="2">
         <v>46056</v>
       </c>
@@ -5584,7 +5630,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="152" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:14">
       <c r="A152" s="2">
         <v>46057</v>
       </c>
@@ -5613,7 +5659,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="153" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:14">
       <c r="A153" s="2">
         <v>46058</v>
       </c>
@@ -5642,7 +5688,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="154" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:14">
       <c r="A154" s="2">
         <v>46059</v>
       </c>
@@ -5674,7 +5720,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="155" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:14">
       <c r="A155" s="2">
         <v>46060</v>
       </c>
@@ -5703,7 +5749,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="156" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:14">
       <c r="A156" s="2">
         <v>46061</v>
       </c>
@@ -5735,7 +5781,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="157" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:14">
       <c r="A157" s="2">
         <v>46062</v>
       </c>
@@ -5764,7 +5810,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="158" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:14">
       <c r="A158" s="2">
         <v>46063</v>
       </c>
@@ -5802,7 +5848,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="159" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:14">
       <c r="A159" s="2">
         <v>46064</v>
       </c>
@@ -5831,7 +5877,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="160" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:14">
       <c r="A160" s="2">
         <v>46065</v>
       </c>
@@ -5860,7 +5906,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="161" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:14">
       <c r="A161" s="2">
         <v>46066</v>
       </c>
@@ -5889,7 +5935,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="162" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:14">
       <c r="A162" s="2">
         <v>46067</v>
       </c>
@@ -5918,7 +5964,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="163" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:14">
       <c r="A163" s="2">
         <v>46068</v>
       </c>
@@ -5950,7 +5996,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="164" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:14">
       <c r="A164" s="2">
         <v>46069</v>
       </c>
@@ -5979,7 +6025,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="165" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:14">
       <c r="A165" s="2">
         <v>46070</v>
       </c>
@@ -6008,7 +6054,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="166" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:14">
       <c r="A166" s="2">
         <v>46071</v>
       </c>
@@ -6040,7 +6086,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="167" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:14">
       <c r="A167" s="2">
         <v>46072</v>
       </c>
@@ -6069,7 +6115,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="168" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:14">
       <c r="A168" s="2">
         <v>46073</v>
       </c>
@@ -6098,7 +6144,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="169" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:14">
       <c r="A169" s="2">
         <v>46074</v>
       </c>
@@ -6127,7 +6173,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="170" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:14">
       <c r="A170" s="2">
         <v>46075</v>
       </c>
@@ -6156,7 +6202,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="171" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:14">
       <c r="A171" s="2">
         <v>46076</v>
       </c>
@@ -6185,7 +6231,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="172" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:14">
       <c r="A172" s="2">
         <v>46077</v>
       </c>
@@ -6214,7 +6260,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="173" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:14">
       <c r="A173" s="2">
         <v>46078</v>
       </c>
@@ -6243,7 +6289,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="174" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:14">
       <c r="A174" s="2">
         <v>46079</v>
       </c>
@@ -6272,7 +6318,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="175" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:14">
       <c r="A175" s="2">
         <v>46080</v>
       </c>
@@ -6301,7 +6347,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="176" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:14">
       <c r="A176" s="2">
         <v>46081</v>
       </c>
@@ -6330,7 +6376,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="177" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:14">
       <c r="A177" s="2">
         <v>46082</v>
       </c>
@@ -6359,7 +6405,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="178" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:14">
       <c r="A178" s="2">
         <v>46083</v>
       </c>
@@ -6388,7 +6434,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="179" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:14">
       <c r="A179" s="2">
         <v>46084</v>
       </c>
@@ -6417,7 +6463,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="180" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:14">
       <c r="A180" s="2">
         <v>46085</v>
       </c>
@@ -6446,7 +6492,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="181" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:14">
       <c r="A181" s="2">
         <v>46086</v>
       </c>
@@ -6482,45 +6528,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:BF4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="6" max="6" width="19.28515625" customWidth="1"/>
-    <col min="7" max="7" width="22.7109375" customWidth="1"/>
-    <col min="28" max="28" width="15.85546875" customWidth="1"/>
-    <col min="29" max="29" width="24.5703125" customWidth="1"/>
-    <col min="30" max="30" width="24.28515625" customWidth="1"/>
-    <col min="31" max="31" width="21.28515625" customWidth="1"/>
-    <col min="32" max="32" width="19.7109375" customWidth="1"/>
-    <col min="33" max="33" width="21.5703125" customWidth="1"/>
-    <col min="34" max="34" width="20.85546875" customWidth="1"/>
-    <col min="35" max="35" width="18.140625" customWidth="1"/>
-    <col min="36" max="36" width="19.7109375" customWidth="1"/>
-    <col min="37" max="37" width="23.5703125" customWidth="1"/>
-    <col min="38" max="38" width="18.85546875" customWidth="1"/>
-    <col min="39" max="39" width="24.42578125" customWidth="1"/>
-    <col min="40" max="40" width="25" customWidth="1"/>
-    <col min="41" max="41" width="21.7109375" customWidth="1"/>
-    <col min="42" max="42" width="20.140625" customWidth="1"/>
-    <col min="43" max="43" width="24.42578125" customWidth="1"/>
-    <col min="44" max="44" width="27.140625" customWidth="1"/>
-    <col min="45" max="45" width="25.42578125" customWidth="1"/>
-    <col min="46" max="46" width="24.5703125" customWidth="1"/>
-    <col min="47" max="47" width="23.42578125" customWidth="1"/>
-    <col min="48" max="48" width="25.28515625" customWidth="1"/>
-    <col min="49" max="49" width="19.7109375" customWidth="1"/>
-    <col min="50" max="50" width="27.140625" customWidth="1"/>
-    <col min="51" max="51" width="29.42578125" customWidth="1"/>
-    <col min="52" max="52" width="29.85546875" customWidth="1"/>
-    <col min="53" max="53" width="32.5703125" customWidth="1"/>
-    <col min="54" max="54" width="28.42578125" customWidth="1"/>
-    <col min="55" max="55" width="23" customWidth="1"/>
-    <col min="56" max="56" width="28.140625" customWidth="1"/>
-    <col min="57" max="57" width="39" customWidth="1"/>
-    <col min="58" max="58" width="38.140625" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:BG4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:59">
       <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
@@ -6695,8 +6706,11 @@
       <c r="BF1" s="1" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="2" spans="1:58" x14ac:dyDescent="0.25">
+      <c r="BG1" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:59">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -6734,13 +6748,13 @@
         <v>45934</v>
       </c>
       <c r="M2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="N2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="P2">
         <v>1000</v>
@@ -6764,7 +6778,7 @@
         <v>50</v>
       </c>
       <c r="W2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="X2">
         <v>1.65</v>
@@ -6835,8 +6849,11 @@
       <c r="BC2">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:58" x14ac:dyDescent="0.25">
+      <c r="BG2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:59">
       <c r="A3" t="s">
         <v>26</v>
       </c>
@@ -6874,13 +6891,13 @@
         <v>45995</v>
       </c>
       <c r="M3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="N3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="P3">
         <v>1000</v>
@@ -6904,7 +6921,7 @@
         <v>50</v>
       </c>
       <c r="W3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="Y3">
         <v>3.3333333333333333E-2</v>
@@ -6972,8 +6989,11 @@
       <c r="BC3">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:58" x14ac:dyDescent="0.25">
+      <c r="BG3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:59">
       <c r="A4" t="s">
         <v>28</v>
       </c>
@@ -7011,13 +7031,13 @@
         <v>46027</v>
       </c>
       <c r="M4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="N4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="P4">
         <v>5000</v>
@@ -7041,7 +7061,7 @@
         <v>50</v>
       </c>
       <c r="W4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="Y4">
         <v>3.3333333333333333E-2</v>
@@ -7144,6 +7164,9 @@
       </c>
       <c r="BF4">
         <v>-2.621083783892991</v>
+      </c>
+      <c r="BG4">
+        <v>1256500</v>
       </c>
     </row>
   </sheetData>
@@ -7153,13 +7176,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F44"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G44"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="3" max="3" width="24.28515625" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
@@ -7170,16 +7193,19 @@
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -7198,8 +7224,11 @@
       <c r="F2">
         <v>210000</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -7218,8 +7247,11 @@
       <c r="F3">
         <v>165000</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -7238,8 +7270,11 @@
       <c r="F4">
         <v>145600</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -7258,8 +7293,11 @@
       <c r="F5">
         <v>140000</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -7278,8 +7316,11 @@
       <c r="F6">
         <v>235200</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -7298,8 +7339,11 @@
       <c r="F7">
         <v>172800</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -7318,8 +7362,11 @@
       <c r="F8">
         <v>110700</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -7338,8 +7385,11 @@
       <c r="F9">
         <v>502200</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -7358,8 +7408,11 @@
       <c r="F10">
         <v>221400</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -7378,8 +7431,11 @@
       <c r="F11">
         <v>175500</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
       <c r="A12" t="s">
         <v>15</v>
       </c>
@@ -7398,8 +7454,11 @@
       <c r="F12">
         <v>197100</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
       <c r="A13" t="s">
         <v>15</v>
       </c>
@@ -7418,8 +7477,11 @@
       <c r="F13">
         <v>216000</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
       <c r="A14" t="s">
         <v>15</v>
       </c>
@@ -7438,8 +7500,11 @@
       <c r="F14">
         <v>164700</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
       <c r="A15" t="s">
         <v>26</v>
       </c>
@@ -7458,8 +7523,11 @@
       <c r="F15">
         <v>114800</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
       <c r="A16" t="s">
         <v>26</v>
       </c>
@@ -7479,7 +7547,7 @@
         <v>423900</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7">
       <c r="A17" t="s">
         <v>26</v>
       </c>
@@ -7499,7 +7567,7 @@
         <v>175500</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7">
       <c r="A18" t="s">
         <v>26</v>
       </c>
@@ -7519,7 +7587,7 @@
         <v>1003600</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7">
       <c r="A19" t="s">
         <v>26</v>
       </c>
@@ -7539,7 +7607,7 @@
         <v>137700</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7">
       <c r="A20" t="s">
         <v>26</v>
       </c>
@@ -7559,7 +7627,7 @@
         <v>392600</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7">
       <c r="A21" t="s">
         <v>26</v>
       </c>
@@ -7579,7 +7647,7 @@
         <v>187200</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7">
       <c r="A22" t="s">
         <v>26</v>
       </c>
@@ -7599,7 +7667,7 @@
         <v>119600</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7">
       <c r="A23" t="s">
         <v>28</v>
       </c>
@@ -7618,8 +7686,11 @@
       <c r="F23">
         <v>390000</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G23" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
       <c r="A24" t="s">
         <v>28</v>
       </c>
@@ -7638,8 +7709,11 @@
       <c r="F24">
         <v>54000</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G24" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
       <c r="A25" t="s">
         <v>28</v>
       </c>
@@ -7658,8 +7732,11 @@
       <c r="F25">
         <v>780000</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G25" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
       <c r="A26" t="s">
         <v>28</v>
       </c>
@@ -7678,8 +7755,11 @@
       <c r="F26">
         <v>232500</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G26" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
       <c r="A27" t="s">
         <v>28</v>
       </c>
@@ -7698,8 +7778,11 @@
       <c r="F27">
         <v>1040000</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G27" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
       <c r="A28" t="s">
         <v>28</v>
       </c>
@@ -7718,8 +7801,11 @@
       <c r="F28">
         <v>1080000</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G28" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
       <c r="A29" t="s">
         <v>28</v>
       </c>
@@ -7738,8 +7824,11 @@
       <c r="F29">
         <v>461700</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G29" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
       <c r="A30" t="s">
         <v>28</v>
       </c>
@@ -7758,8 +7847,11 @@
       <c r="F30">
         <v>625000</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G30" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
       <c r="A31" t="s">
         <v>28</v>
       </c>
@@ -7778,8 +7870,11 @@
       <c r="F31">
         <v>297000</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G31" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
       <c r="A32" t="s">
         <v>28</v>
       </c>
@@ -7798,8 +7893,11 @@
       <c r="F32">
         <v>1021800</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G32" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
       <c r="A33" t="s">
         <v>28</v>
       </c>
@@ -7818,8 +7916,11 @@
       <c r="F33">
         <v>757500</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G33" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
       <c r="A34" t="s">
         <v>28</v>
       </c>
@@ -7838,8 +7939,11 @@
       <c r="F34">
         <v>500000</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G34" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
       <c r="A35" t="s">
         <v>28</v>
       </c>
@@ -7858,8 +7962,11 @@
       <c r="F35">
         <v>137500</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G35" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
       <c r="A36" t="s">
         <v>28</v>
       </c>
@@ -7878,8 +7985,11 @@
       <c r="F36">
         <v>10000</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G36" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
       <c r="A37" t="s">
         <v>28</v>
       </c>
@@ -7898,8 +8008,11 @@
       <c r="F37">
         <v>1150000</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G37" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
       <c r="A38" t="s">
         <v>28</v>
       </c>
@@ -7918,8 +8031,11 @@
       <c r="F38">
         <v>81000</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G38" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
       <c r="A39" t="s">
         <v>28</v>
       </c>
@@ -7938,8 +8054,11 @@
       <c r="F39">
         <v>137500</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G39" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
       <c r="A40" t="s">
         <v>28</v>
       </c>
@@ -7958,8 +8077,11 @@
       <c r="F40">
         <v>1125000</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G40" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
       <c r="A41" t="s">
         <v>28</v>
       </c>
@@ -7978,8 +8100,11 @@
       <c r="F41">
         <v>375000</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G41" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
       <c r="A42" t="s">
         <v>28</v>
       </c>
@@ -7998,8 +8123,11 @@
       <c r="F42">
         <v>5000</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G42" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7">
       <c r="A43" t="s">
         <v>28</v>
       </c>
@@ -8018,8 +8146,11 @@
       <c r="F43">
         <v>1000000</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G43" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
       <c r="A44" t="s">
         <v>28</v>
       </c>
@@ -8037,6 +8168,9 @@
       </c>
       <c r="F44">
         <v>1052500</v>
+      </c>
+      <c r="G44" t="s">
+        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>